<commit_message>
chore(ledger): feedback Diana PANTHER EXPRESS 2026-08-03
R-015 VIGENTE (Type of Trucker segun operacion), R-002 refinada (filings
siempre Yes + State/Federal segun radio), R-078 anotada (alcance GEICO
en duda), R-085 nueva (zip vehiculo = physical address, Ambos),
R-086 nueva (PDF con fecha AAAA-MM-DD).

Co-Authored-By: Claude Fable 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H3Ntj2k8bsY6g2HVLh84hr
</commit_message>
<xml_diff>
--- a/config/mga_decision_rules.xlsx
+++ b/config/mga_decision_rules.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -565,7 +565,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes siempre. Tipo de filing según radio de operación: intraestatal → State, interestatal → Federal</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>USDOT 9648609</t>
+          <t>USDOT 9648609; PANTHER EXPRESS 4514637</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>commit c53f4eb. El radio vive en MoreAboutBusiness (la semilla del plan decía RATES). El '&lt;60 días' del USDOT es R-009.</t>
+          <t>commit c53f4eb. El radio vive en MoreAboutBusiness (la semilla del plan decía RATES). El '&lt;60 días' del USDOT es R-009. || 2026-08-03 Diana (PANTHER): filings siempre Yes; estatal o federal se elige según el radio del cliente. En PANTHER quedaron marcados Federal Liability + MCS-90 + State a la vez — verificar si los marca el bot o vienen pre-marcados por Progressive.</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,6 @@
           <t>Negocio</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>VIGENTE</t>
@@ -881,7 +880,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1033,7 +1031,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1081,7 +1078,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1181,7 +1177,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1221,27 +1216,27 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>'General Freight / Other'</t>
+          <t>Según la operación real del cliente (flatbed → Flatbed, dry van → Dry Van, reefer → Refrigerated, etc.). 'General Freight / Other' solo como último recurso sin señal de operación</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Default técnico</t>
+          <t>Negocio (Diana)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>JUAREZ LOGISTICS</t>
+          <t>JUAREZ LOGISTICS; PANTHER EXPRESS 4514637 (CA117638002)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>EN-DUDA</t>
+          <t>VIGENTE</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>business_info_page.py:517,573-578 — resolve_choice ya lo registra en el ledger (DEFAULTED)</t>
+          <t>business_info_page.py:517,573-578 — resolve_choice ya lo registra en el ledger (DEFAULTED) || 2026-08-03 Diana (PANTHER): la clasificación debe corresponder a la operación; ya lo había pedido en correos anteriores. Fix pendiente en código.</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1276,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1329,7 +1323,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1429,7 +1422,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1477,7 +1469,6 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1525,7 +1516,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1573,7 +1563,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1829,7 +1818,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1877,7 +1865,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1925,7 +1912,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -1973,7 +1959,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -2073,7 +2058,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -2121,7 +2105,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -2429,7 +2412,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -2477,7 +2459,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -2629,7 +2610,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -2729,7 +2709,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -2829,7 +2808,6 @@
           <t>Negocio</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
           <t>VIGENTE</t>
@@ -2877,7 +2855,6 @@
           <t>Negocio</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
           <t>VIGENTE</t>
@@ -3029,7 +3006,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -3077,7 +3053,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -3125,7 +3100,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -3277,7 +3251,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -3325,7 +3298,6 @@
           <t>Negocio</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
           <t>VIGENTE</t>
@@ -3373,7 +3345,6 @@
           <t>Negocio</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
           <t>VIGENTE</t>
@@ -3473,7 +3444,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -3521,7 +3491,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -3777,7 +3746,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -3825,7 +3793,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -3977,7 +3944,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4025,7 +3991,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4073,7 +4038,6 @@
           <t>Negocio</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr">
         <is>
           <t>VIGENTE</t>
@@ -4121,7 +4085,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4169,7 +4132,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4217,7 +4179,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4265,7 +4226,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4313,7 +4273,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4361,7 +4320,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4369,7 +4327,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>field_mapper.py:617 + additional_business_page.py:193-197. INCONSISTENCIA con R-002: en Progressive va Yes (Diana).</t>
+          <t>field_mapper.py:617 + additional_business_page.py:193-197. INCONSISTENCIA con R-002: en Progressive va Yes (Diana). || 2026-08-03 Diana (PANTHER): 'los filings siempre debe ir sí' (dicho en contexto Progressive); confirmar alcance GEICO en la sesión — sigue EN-DUDA.</t>
         </is>
       </c>
     </row>
@@ -4409,7 +4367,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
       <c r="I80" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4457,7 +4414,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4505,7 +4461,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4605,7 +4560,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4653,7 +4607,6 @@
           <t>Default técnico</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
           <t>EN-DUDA</t>
@@ -4662,6 +4615,110 @@
       <c r="J85" t="inlineStr">
         <is>
           <t>final_details_page.py:83-86</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>R-085</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Add Vehicle (Prog) / Step 3 Vehicles (GEICO)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Zip donde se ubica el vehículo (garaging)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Siempre</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Zip de la PHYSICAL address del BlueQuote — nunca la mailing</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Negocio (Diana)</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>PANTHER EXPRESS 4514637 (CA117638002)</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>VIGENTE</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>2026-08-03: el bot usó 77095 (mailing, 7834 Maple Brook Ln) en vez de 77041 (physical, 7800 Wright Rd). Fix pendiente en extractor/field_mapper de ambos módulos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>R-086</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Progressive</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>RATES → Print/Send (PDF)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Nombre de archivo del quote PDF</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Al guardar la cotización descargada</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Nombre con fecha AAAA-MM-DD (año, mes, día) — no el nombre por defecto de la página</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Negocio (Diana)</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>PANTHER EXPRESS 4514637</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>VIGENTE</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>2026-08-03 (2º correo). Aplica al feature de descarga de PDF (spec 2026-07-06, aún no implementado). El PDF va en la subcarpeta 'quotes' del cliente (ver plan alcance D).</t>
         </is>
       </c>
     </row>
@@ -4689,9 +4746,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -4713,9 +4768,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -4751,9 +4804,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -4796,9 +4847,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -4813,9 +4862,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -4837,9 +4884,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(progressive): manejar el interstitial Filing/Proof of Insurance (R-087)
Los ultimos 3 jobs (PANTHER CA117638002, ALTIMO CA117637552, G&E
CA117642658) morian esperando el premium de RATES parados en esta
pagina, que Progressive muestra desde que R-002 responde Yes a los
filings. Nuevo FilingProofPage: radio include-all-vehicles=Yes,
Filings Needed se dejan como Progressive los pre-marca (SAFER),
Continue con fallback por heading si el pageName no cambia. Todo
queda en el ledger bajo R-087 (EN-DUDA: State vs Federal por radio
pendiente de sesion con Diana). Wire en quote_flow step 6.5.

Pendiente: validacion live con la proxima Submission real.

Co-Authored-By: Claude Fable 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H3Ntj2k8bsY6g2HVLh84hr
</commit_message>
<xml_diff>
--- a/config/mga_decision_rules.xlsx
+++ b/config/mga_decision_rules.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4719,6 +4719,58 @@
       <c r="J87" t="inlineStr">
         <is>
           <t>2026-08-03 (2º correo). Aplica al feature de descarga de PDF (spec 2026-07-06, aún no implementado). El PDF va en la subcarpeta 'quotes' del cliente (ver plan alcance D).</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>R-087</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Progressive</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Filing/Proof of Insurance (interstitial)</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Radio 'include all vehicles' + checkboxes 'Filings Needed'</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Aparece entre BUSINESS y RATES cuando R-002=Yes (cliente con autoridad)</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Radio=Yes siempre; checkboxes de Filings Needed se dejan como Progressive los pre-marca (SAFER)</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Default técnico</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>PANTHER EXPRESS 4514637 (CA117638002)</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>EN-DUDA</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>2026-08-03: Diana pide elegir State vs Federal según el radio de operación — falta el criterio exacto (umbral de millas / tipo de autoridad) para automatizarlo; validar en sesión. Página descubierta porque los 3 últimos jobs Progressive morían aquí esperando el premium.</t>
         </is>
       </c>
     </row>
@@ -4746,7 +4798,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -4768,7 +4819,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -4804,7 +4854,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -4847,7 +4896,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -4862,7 +4910,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -4884,7 +4931,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(live): R-088 effective date vencida, R-089 carrier NEW BUSINESS, R-090 DBA individual
Primera corrida live post-despliegue (T&S Logistics 9731476):
- R-088: la effective date del subject ya habia vencido y Progressive la
  rechaza ("cannot be less than <hoy>") -> clamp a HOY en el orquestador
- R-089: current_carrier='NEW BUSINESS' es sentinel de negocio nuevo, no un
  carrier -> ahora implica new venture (antes forzaba establecido, invertido)
- R-090: Individual/Sole Prop no renderiza el radio de Business Name ->
  el nombre comercial va a 'DBA Name' sin quemar timeouts

Ledger: 3 reglas nuevas EN-DUDA. Suite: 714 passed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EnPQCAeqczT2RukAVZ2oPS
</commit_message>
<xml_diff>
--- a/config/mga_decision_rules.xlsx
+++ b/config/mga_decision_rules.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4776,6 +4776,162 @@
       <c r="J88" t="inlineStr">
         <is>
           <t>2026-08-03: Diana pide elegir State vs Federal según el radio de operación — falta el criterio exacto (umbral de millas / tipo de autoridad) para automatizarlo; validar en sesión. Página descubierta porque los 3 últimos jobs Progressive morían aquí esperando el premium. || 2026-08-04: criterio validado por Diana. El MVP actual (dejar lo pre-marcado) queda como fallback; fix del criterio pendiente en código.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>R-088</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>START (Prog) / inicio (GEICO)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Effective date</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>La fecha del subject ya vencio</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Se cotiza con HOY (los portales exigen &gt;= hoy; Progressive: "cannot be less than"). El log deja rastro.</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Default tecnico</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>T&amp;S LOGISTICS 9731476 (08/05 vencida)</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>EN-DUDA</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Validar con Diana: cotizar con hoy vs devolver a ventas por fecha nueva.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>R-089</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Orquestador (pre-encolado)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>is_new_venture</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Blue Quote con current_carrier=NEW BUSINESS/NEW VENTURE</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Es un sentinel de negocio SIN aseguradora -&gt; se trata como NEW VENTURE (antes se invertia: lo tomaba como carrier real y forzaba establecido).</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Default tecnico</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>T&amp;S LOGISTICS 9731476</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>EN-DUDA</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Semantica de la Blue Quote; confirmar con Diana que no hay caso contrario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>R-090</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>PROGRESSIVE</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Business Name / DBA</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Entidad Individual / Sole Proprietor (no renderiza el radio de Business Name)</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>El nombre comercial de la Blue Quote se pone en "DBA Name" (opcional); el named insured es el owner.</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Default tecnico</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>T&amp;S LOGISTICS 9731476</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>EN-DUDA</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Confirmar con Diana que el trade name debe ir como DBA en sole props.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: R-092 (New Venture sin USDOT) + R-091 en el registro de reglas
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EnPQCAeqczT2RukAVZ2oPS
</commit_message>
<xml_diff>
--- a/config/mga_decision_rules.xlsx
+++ b/config/mga_decision_rules.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J91"/>
+  <dimension ref="A1:J93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4932,6 +4932,110 @@
       <c r="J91" t="inlineStr">
         <is>
           <t>Confirmar con Diana que el trade name debe ir como DBA en sole props.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>R-091</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>GEICO</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Step 1 Business Class &amp; USDOT</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Current GEICO commercial auto policy</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Pregunta nueva del dashboard rediseñado; Step 1 la muestra siempre.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Default tecnico</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>G&amp;E HAULING LLC</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>EN-DUDA</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Ventas manda submissions de negocio NUEVO; si ya tuviera poliza GEICO vigente seria renovacion. Confirmar con Diana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>R-092</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>PROGRESSIVE + GEICO</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>START / Step 1</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Does the customer have a USDOT Number?</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>New Venture: la Blue Quote trae USDOT N/A. Antes se abortaba la cotizacion.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Not Yet (el cliente aplico / aplicara). NUNCA "No".</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Diana 2026-08-06</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>DIANA CAROLINA GARCIA OSORIO</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>VIGENTE</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Diana: "Solo funciona Progressive y Geico para ese tipo de clientes / no hay necesidad de verificar el USDOT". Se elige Not Yet y no No porque un New Venture de trucking SI va a tener USDOT; decir que nunca lo tendra seria falso ante el carrier y cambia el rating. Verificado live que ambos portales dejan cotizar sin USDOT. FALTA validacion live end-to-end.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: changelog de la ola 2026-08-10 + R-093..R-096 en el registro
R-093 (plataformas cuentan) y R-094 (adjuntos) quedan VIGENTE.
R-096 (dos limites de AL) queda EN-DUDA: hay que definir si el bot cotiza los
dos por si mismo.
R-095 (condados) VIGENTE con la salvedad de Beaumont ciudad vs. condado.

Incluye dos hallazgos operativos de la misma revision que NO son de la ola:
el contenedor lleva 2 dias parado (exit 137 pero OOMKilled=false -> lo
pararon, no crasheo) y el guard esta descartando submissions originales de
remitentes dados de alta solo en el grupo new_venture.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EnPQCAeqczT2RukAVZ2oPS
</commit_message>
<xml_diff>
--- a/config/mga_decision_rules.xlsx
+++ b/config/mga_decision_rules.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J93"/>
+  <dimension ref="A1:J97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5036,6 +5036,214 @@
       <c r="J93" t="inlineStr">
         <is>
           <t>Diana: "Solo funciona Progressive y Geico para ese tipo de clientes / no hay necesidad de verificar el USDOT". Se elige Not Yet y no No porque un New Venture de trucking SI va a tener USDOT; decir que nunca lo tendra seria falso ante el carrier y cambia el rating. Verificado live que ambos portales dejan cotizar sin USDOT. FALTA validacion live end-to-end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>R-093</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>PROGRESSIVE + GEICO + BERKSHIRE</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Correo de analisis</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>MGAs elegibles (conteo y listado)</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Las MGAs de portal se evaluaban pero se excluian de la lista y del contador: el correo decia '0 ELEGIBLE(S)' y 'Ninguna MGA califica' al lado de un bloque que las daba por elegibles.</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Las MGAs de portal cuentan y se listan como elegibles, marcadas como 'plataforma en linea'. Berkshire entra al grupo: los documentos se cargan en su portal, no se reenvian por correo, asi que el guard de adjuntos no la baja a no elegible.</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Diana 2026-08-10</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>T&amp;S LOGISTICS 9731476</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>VIGENTE</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Diana: "en MGA elegible si aplica con Progressive, Geico y Berkshire mas sin embargo, no lo toma en cuenta" + "anadir berkshire es una plataforma en linea". Reemplaza el criterio de 2026-06-25 (un decline del RPA sigue mandando en la seccion RPA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>R-094</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>TODAS</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Correo de analisis</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Adjuntos reenviados a negocio</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Gmail nombra 'noname' a toda imagen inline (firmas del remitente). Las 5 del correo de T&amp;S se escribieron sobre la misma ruta y el analisis salio con 5 copias del mismo logo de 7 KB.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Las imagenes inline de la firma no se reenvian. Los documentos del cliente conservan su nombre original (dice el limite pedido) y si se repite se desambigua con sufijo, nunca se pisa.</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Diana 2026-08-10</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>T&amp;S LOGISTICS 9731476</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>VIGENTE</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Diana: "al nombrarlo va a causar confusion... eso se debe organizar" + "nombrar bien los documentos".</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>R-095</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>AMWINS</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Rule engine</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Condado del zip code physical</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>El programa no aplica en ciertos condados de Texas; antes no se miraba el condado.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Inelegible si el zip PHYSICAL cae en Brazoria, Fort Bend, Galveston, Harris, Montgomery, Hidalgo, Starr, Cameron o Beaumont. Un zip que no se puede mapear AVISA para revision manual, no bloquea.</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Diana 2026-08-10</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>T&amp;S LOGISTICS 9731476</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>VIGENTE</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>PENDIENTE con Diana: Beaumont es CIUDAD (condado Jefferson). Se bloquean los zips de la ciudad; confirmar si queria el condado entero (Port Arthur, Nederland, Groves, Port Neches). El mapa zip-&gt;condado de modules/tx_counties.py cubre solo los condados bloqueados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>R-096</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>PROGRESSIVE + GEICO</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>RATES / coberturas</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Limite de Auto Liability pedido</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>El agente pidio DOS limites: $1M CSL en la Blue Quote y $750K en una segunda Blue Quote y en el cuerpo del correo ('POR FAVOR SOLICITAR UNA QUOTE DE $750,000 TAMBIEN'). El clasificador descarto la segunda Blue Quote como duplicada y el pedido se perdio.</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Se cotiza el limite principal y el/los adicionales salen como aviso destacado en el analisis para hacerlos a mano.</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Diana 2026-08-10</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>T&amp;S LOGISTICS 9731476</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>EN-DUDA</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>PENDIENTE con Diana: definir si el bot debe cotizar los dos limites por si mismo (un job por MGA+limite) en vez de solo avisar.</t>
         </is>
       </c>
     </row>

</xml_diff>